<commit_message>
Sprint Review 1: infraestructura al Sprint 6 y nada de la app como realizado
- Decision 5 en el acta: SMTP, almacenamiento de archivos, clave de Google
  Maps, push y HTTPS de la API los provee Codigo Creativo en el Sprint 6
  (T-6301..T-6305 en el Sprint Backlog S6). Impedimentos 1, 2 y 4 en gestion;
  HU-004 pasa a En revision.
- S6: todo lo movido de la app queda Por hacer (lo adelantado es MVP interno).
- Retrospective: acuerdo A5 y DoD ajustados.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fase 2/SIGMA_Bitacora_Daily_Scrum.xlsx
+++ b/Fase 2/SIGMA_Bitacora_Daily_Scrum.xlsx
@@ -12787,12 +12787,12 @@
       </c>
       <c r="I5" s="28" t="inlineStr">
         <is>
-          <t>Pendiente: conseguir host, puerto, usuario y clave del servidor de correo. El código ya está hecho y no requiere cambios.</t>
+          <t>Reprogramado al Sprint 6 en la Sprint Review 1 (15-09-2026): toda la infraestructura y los servicios externos se concentran ahí y los provee Código Creativo (T-6301). HU-004 queda construida y en revisión; el criterio del correo se verifica en el Sprint 6.</t>
         </is>
       </c>
       <c r="J5" s="22" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>En gestión</t>
         </is>
       </c>
       <c r="K5" s="23" t="n"/>
@@ -12840,12 +12840,12 @@
       </c>
       <c r="I6" s="28" t="inlineStr">
         <is>
-          <t>Las pantallas ya avisan en pantalla y esconden el formulario en vez de fallar al guardar. Hay que decidir proveedor y crear el servicio.</t>
+          <t>Reprogramado al Sprint 6 en la Sprint Review 1 (15-09-2026), junto con las evidencias desde terreno (HU-140/141): Código Creativo decide proveedor y levanta el servicio (T-6302). Las pantallas web siguen avisando y escondiendo el formulario mientras tanto.</t>
         </is>
       </c>
       <c r="J6" s="22" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>En gestión</t>
         </is>
       </c>
       <c r="K6" s="23" t="n"/>
@@ -12946,12 +12946,12 @@
       </c>
       <c r="I8" s="28" t="inlineStr">
         <is>
-          <t>Pendiente: entrar a la consola de Google Cloud y verificar restricción por referrer y APIs habilitadas.</t>
+          <t>Reprogramado al Sprint 6 en la Sprint Review 1 (15-09-2026): restricción de la clave en la consola de Google Cloud (T-6303).</t>
         </is>
       </c>
       <c r="J8" s="22" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>En gestión</t>
         </is>
       </c>
       <c r="K8" s="23" t="n"/>

</xml_diff>

<commit_message>
Planillas sincronizadas con el avance de Catalina en el Sprint 5
Product Backlog: HU-142 En revisión, HU-143 En curso. Pendientes: fuera
las 11 tareas terminadas (S5 queda en 40 tareas y 16,75 h; Catalina 2,75 h).
Bitácora: los dailies de Catalina del 04 al 10-11 registran HU-142 y lo
hecho de HU-143, y el cierre del Sprint 5 lo refleja.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fase 2/SIGMA_Bitacora_Daily_Scrum.xlsx
+++ b/Fase 2/SIGMA_Bitacora_Daily_Scrum.xlsx
@@ -883,7 +883,7 @@
       </c>
       <c r="C17" s="29" t="inlineStr">
         <is>
-          <t>1.1 · 22-09-2026 · Sprints 1 a 5 con registro diario</t>
+          <t>1.2 · 12-10-2026 · Sprints 1 a 5 con registro diario; avance de Catalina en el Sprint 5 (HU-142 y HU-143)</t>
         </is>
       </c>
     </row>
@@ -11823,12 +11823,12 @@
       </c>
       <c r="I141" s="37" t="inlineStr">
         <is>
-          <t>Sin avance de desarrollo.</t>
+          <t>Tomé HU-142 y HU-143, las dos sobre Archivo_Vinculo. Revisé el modelo: no hace falta tabla nueva, la galería del equipo sale por la orden, y una imagen de referencia se reconoce por su destino (actividad del plan o ítem de pauta), no por avi_es_referencia. Dejé los índices de la galería y la semilla de prueba (BD/429).</t>
         </is>
       </c>
       <c r="J141" s="37" t="inlineStr">
         <is>
-          <t>Subir HU-082.</t>
+          <t>Escribir SEL_ARCHIVO_VINCULO para las dos galerías.</t>
         </is>
       </c>
       <c r="K141" s="37" t="inlineStr">
@@ -11838,12 +11838,12 @@
       </c>
       <c r="L141" s="37" t="inlineStr">
         <is>
-          <t>HU-091, HU-092, HU-097, HU-101</t>
+          <t>HU-142, HU-143</t>
         </is>
       </c>
       <c r="M141" s="37" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>T-5250, T-5252, T-5253, T-5261</t>
         </is>
       </c>
       <c r="N141" s="37" t="inlineStr">
@@ -12048,12 +12048,12 @@
       </c>
       <c r="I144" s="37" t="inlineStr">
         <is>
-          <t>Sin avance de desarrollo.</t>
+          <t>SEL_ARCHIVO_VINCULO: un solo SP para la galería de una orden (por paso y momento) y la de un equipo (todas sus órdenes, por fecha), con filtros y paginación por parámetros, sin firma ni lo de otro cliente (BD/430). Probado contra la semilla.</t>
         </is>
       </c>
       <c r="J144" s="37" t="inlineStr">
         <is>
-          <t>Subir HU-082.</t>
+          <t>Llevar la galería a la ficha de la orden y del activo.</t>
         </is>
       </c>
       <c r="K144" s="37" t="inlineStr">
@@ -12063,12 +12063,12 @@
       </c>
       <c r="L144" s="37" t="inlineStr">
         <is>
-          <t>HU-091, HU-092, HU-097, HU-101</t>
+          <t>HU-142</t>
         </is>
       </c>
       <c r="M144" s="37" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>T-5251</t>
         </is>
       </c>
       <c r="N144" s="37" t="inlineStr">
@@ -12273,12 +12273,12 @@
       </c>
       <c r="I147" s="37" t="inlineStr">
         <is>
-          <t>Sin avance de desarrollo.</t>
+          <t>La galería quedó dentro de la ficha de la OT (pestaña Pasos, por paso y momento, con visor para ampliar y descargar) y de la ficha del activo, que ahora suma las fotos de los pasos. Las referencias salen aparte, en «Cómo debe quedar» y en el chip «Referencias». Los métodos exigen el permiso y el SP filtra por cliente.</t>
         </is>
       </c>
       <c r="J147" s="37" t="inlineStr">
         <is>
-          <t>Subir HU-082.</t>
+          <t>Publicar la galería en la API para la app.</t>
         </is>
       </c>
       <c r="K147" s="37" t="inlineStr">
@@ -12288,12 +12288,12 @@
       </c>
       <c r="L147" s="37" t="inlineStr">
         <is>
-          <t>HU-091, HU-092, HU-097, HU-101</t>
+          <t>HU-142, HU-143</t>
         </is>
       </c>
       <c r="M147" s="37" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>T-5256, T-5258</t>
         </is>
       </c>
       <c r="N147" s="37" t="inlineStr">
@@ -12498,12 +12498,12 @@
       </c>
       <c r="I150" s="37" t="inlineStr">
         <is>
-          <t>Sin avance de desarrollo.</t>
+          <t>GET /api/archivo-vinculos: la misma galería para la app, con el mismo SP que la web, paginada en el servidor y con caché corta de 30 s. Probado por HTTP con un usuario técnico de Hamburgo, incluida una orden de otro cliente (0 filas).</t>
         </is>
       </c>
       <c r="J150" s="37" t="inlineStr">
         <is>
-          <t>Preparar la aceptación de lo de Bryan.</t>
+          <t>Pruebas y documentación de HU-142; preparar la aceptación de lo de Bryan.</t>
         </is>
       </c>
       <c r="K150" s="37" t="inlineStr">
@@ -12513,17 +12513,17 @@
       </c>
       <c r="L150" s="37" t="inlineStr">
         <is>
-          <t>HU-091, HU-092, HU-097, HU-101</t>
+          <t>HU-142</t>
         </is>
       </c>
       <c r="M150" s="37" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>T-5254, T-5255</t>
         </is>
       </c>
       <c r="N150" s="37" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="O150" s="22" t="n"/>
@@ -12723,12 +12723,12 @@
       </c>
       <c r="I153" s="37" t="inlineStr">
         <is>
-          <t>Recorrí las ocho historias de Bryan contra sus criterios; la validación funcional queda pendiente, así que se van En revisión. De lo mío no entregué nada en este Sprint.</t>
+          <t>Recorrí las ocho historias de Bryan contra sus criterios; la validación funcional queda pendiente, así que se van En revisión. De lo mío: HU-142 con sus dos criterios probados y documentada, queda En revisión (el consumo desde la app pasa al Sprint 6). HU-143 queda a medias: falta adjuntar la referencia desde la actividad del plan y el ítem de pauta.</t>
         </is>
       </c>
       <c r="J153" s="37" t="inlineStr">
         <is>
-          <t>Cerrar HU-082, HU-091 y HU-097 antes de que empiece el Sprint 6.</t>
+          <t>Terminar HU-143 y cerrar HU-082, HU-091 y HU-097 antes de que empiece el Sprint 6.</t>
         </is>
       </c>
       <c r="K153" s="37" t="inlineStr">
@@ -12738,17 +12738,17 @@
       </c>
       <c r="L153" s="37" t="inlineStr">
         <is>
-          <t>Sprint 5 completo</t>
+          <t>HU-142, HU-143</t>
         </is>
       </c>
       <c r="M153" s="37" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>T-5259, T-5260</t>
         </is>
       </c>
       <c r="N153" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="O153" s="22" t="n"/>
@@ -12798,7 +12798,7 @@
       </c>
       <c r="I154" s="37" t="inlineStr">
         <is>
-          <t>Facilité la Sprint Review. Se recorrieron las ocho historias de Bryan y quedan En revisión, a la espera de la validación de la Product Owner; doce historias de App del Sprint se van al Sprint 6 por el cambio de alcance. De lo mío y de lo de Catalina no entró nada.</t>
+          <t>Facilité la Sprint Review. Se recorrieron las ocho historias de Bryan y quedan En revisión, a la espera de la validación de la Product Owner; doce historias de App del Sprint se van al Sprint 6 por el cambio de alcance. De Catalina, HU-142 queda En revisión y HU-143 a medias; de lo mío no entró nada.</t>
         </is>
       </c>
       <c r="J154" s="37" t="inlineStr">
@@ -12834,7 +12834,7 @@
       </c>
       <c r="Q154" s="37" t="inlineStr">
         <is>
-          <t>CIERRE DEL SPRINT 5. Se recorren las ocho historias de Bryan (89 tareas), que quedan En revisión hasta la validación de la PO. Se reconoce el desbalance: de 313 tareas del Sprint, 89 son de Bryan terminadas y ninguna de Emilio o Catalina. El equipo acuerda que el Sprint 6 se planifica sobre lo que cada uno puede sostener de verdad, y que las historias bloqueantes del Sprint 4 (HU-082, HU-091, HU-097) entran primero. Dejamos constancia de algo que se ve en las fechas: vamos adelantados respecto del calendario. SIGMA son 785 puntos, 138 historias y 20 épicas para un equipo de tres, y la única forma de absorber ese alcance fue adelantar construcción: lo que aquí se registra en la ventana del Sprint 4 y del Sprint 5 quedó construido y verificado contra la base entre el 11 y el 14 de septiembre. El registro mantiene el calendario planificado para no romper la trazabilidad con el Sprint Backlog, el burndown y los informes de prueba. REPARTO PARA TERMINAR EL SPRINT 5: cada historia la hace UNA persona de punta a punta —desarrollo, pruebas, documentación y validación—, y las que tocan el mismo código van juntas: Bryan HU-117 y HU-125 (la orden), Catalina HU-142 y HU-143 (Archivo_Vinculo), Emilio HU-131 y HU-162.</t>
+          <t>CIERRE DEL SPRINT 5. Se recorren las ocho historias de Bryan (89 tareas), que quedan En revisión hasta la validación de la PO. Se reconoce el desbalance: de 313 tareas del Sprint, 89 son de Bryan terminadas, 11 de Catalina (HU-142 y la revisión del modelo de HU-143) y ninguna de Emilio. El equipo acuerda que el Sprint 6 se planifica sobre lo que cada uno puede sostener de verdad, y que las historias bloqueantes del Sprint 4 (HU-082, HU-091, HU-097) entran primero. Dejamos constancia de algo que se ve en las fechas: vamos adelantados respecto del calendario. SIGMA son 785 puntos, 138 historias y 20 épicas para un equipo de tres, y la única forma de absorber ese alcance fue adelantar construcción: lo que aquí se registra en la ventana del Sprint 4 y del Sprint 5 quedó construido y verificado contra la base entre el 11 y el 14 de septiembre. El registro mantiene el calendario planificado para no romper la trazabilidad con el Sprint Backlog, el burndown y los informes de prueba. REPARTO PARA TERMINAR EL SPRINT 5: cada historia la hace UNA persona de punta a punta —desarrollo, pruebas, documentación y validación—, y las que tocan el mismo código van juntas: Bryan HU-117 y HU-125 (la orden), Catalina termina HU-143 (Archivo_Vinculo), la que le queda de las dos que tomó, Emilio HU-131 y HU-162.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Planillas: HU-143 terminada y en revisión (S5, Product Backlog, Pendientes y bitácora)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fase 2/SIGMA_Bitacora_Daily_Scrum.xlsx
+++ b/Fase 2/SIGMA_Bitacora_Daily_Scrum.xlsx
@@ -883,7 +883,7 @@
       </c>
       <c r="C17" s="29" t="inlineStr">
         <is>
-          <t>1.2 · 12-10-2026 · Sprints 1 a 5 con registro diario; avance de Catalina en el Sprint 5 (HU-142 y HU-143)</t>
+          <t>1.3 · 12-10-2026 · Sprints 1 a 5 con registro diario; HU-142 y HU-143 de Catalina En revisión</t>
         </is>
       </c>
     </row>
@@ -12723,12 +12723,12 @@
       </c>
       <c r="I153" s="37" t="inlineStr">
         <is>
-          <t>Recorrí las ocho historias de Bryan contra sus criterios; la validación funcional queda pendiente, así que se van En revisión. De lo mío: HU-142 con sus dos criterios probados y documentada, queda En revisión (el consumo desde la app pasa al Sprint 6). HU-143 queda a medias: falta adjuntar la referencia desde la actividad del plan y el ítem de pauta.</t>
+          <t>Recorrí las ocho historias de Bryan contra sus criterios; la validación funcional queda pendiente, así que se van En revisión. De lo mío: HU-142 con sus dos criterios probados y documentada, queda En revisión (el consumo desde la app pasa al Sprint 6). HU-143 también queda En revisión: la imagen de referencia se adjunta en el cajón de la actividad y en el ítem de la pauta, y se ve en la OT y junto a la pregunta de la inspección.</t>
         </is>
       </c>
       <c r="J153" s="37" t="inlineStr">
         <is>
-          <t>Terminar HU-143 y cerrar HU-082, HU-091 y HU-097 antes de que empiece el Sprint 6.</t>
+          <t>Cerrar HU-082, HU-091 y HU-097 antes de que empiece el Sprint 6.</t>
         </is>
       </c>
       <c r="K153" s="37" t="inlineStr">
@@ -12743,7 +12743,7 @@
       </c>
       <c r="M153" s="37" t="inlineStr">
         <is>
-          <t>T-5259, T-5260</t>
+          <t>T-5259, T-5260, T-5262 a T-5276</t>
         </is>
       </c>
       <c r="N153" s="37" t="inlineStr">
@@ -12798,7 +12798,7 @@
       </c>
       <c r="I154" s="37" t="inlineStr">
         <is>
-          <t>Facilité la Sprint Review. Se recorrieron las ocho historias de Bryan y quedan En revisión, a la espera de la validación de la Product Owner; doce historias de App del Sprint se van al Sprint 6 por el cambio de alcance. De Catalina, HU-142 queda En revisión y HU-143 a medias; de lo mío no entró nada.</t>
+          <t>Facilité la Sprint Review. Se recorrieron las ocho historias de Bryan y quedan En revisión, a la espera de la validación de la Product Owner; doce historias de App del Sprint se van al Sprint 6 por el cambio de alcance. De Catalina, HU-142 y HU-143 quedan En revisión; de lo mío no entró nada.</t>
         </is>
       </c>
       <c r="J154" s="37" t="inlineStr">
@@ -12834,7 +12834,7 @@
       </c>
       <c r="Q154" s="37" t="inlineStr">
         <is>
-          <t>CIERRE DEL SPRINT 5. Se recorren las ocho historias de Bryan (89 tareas), que quedan En revisión hasta la validación de la PO. Se reconoce el desbalance: de 313 tareas del Sprint, 89 son de Bryan terminadas, 11 de Catalina (HU-142 y la revisión del modelo de HU-143) y ninguna de Emilio. El equipo acuerda que el Sprint 6 se planifica sobre lo que cada uno puede sostener de verdad, y que las historias bloqueantes del Sprint 4 (HU-082, HU-091, HU-097) entran primero. Dejamos constancia de algo que se ve en las fechas: vamos adelantados respecto del calendario. SIGMA son 785 puntos, 138 historias y 20 épicas para un equipo de tres, y la única forma de absorber ese alcance fue adelantar construcción: lo que aquí se registra en la ventana del Sprint 4 y del Sprint 5 quedó construido y verificado contra la base entre el 11 y el 14 de septiembre. El registro mantiene el calendario planificado para no romper la trazabilidad con el Sprint Backlog, el burndown y los informes de prueba. REPARTO PARA TERMINAR EL SPRINT 5: cada historia la hace UNA persona de punta a punta —desarrollo, pruebas, documentación y validación—, y las que tocan el mismo código van juntas: Bryan HU-117 y HU-125 (la orden), Catalina termina HU-143 (Archivo_Vinculo), la que le queda de las dos que tomó, Emilio HU-131 y HU-162.</t>
+          <t>CIERRE DEL SPRINT 5. Se recorren las ocho historias de Bryan (89 tareas), que quedan En revisión hasta la validación de la PO. Se reconoce el desbalance: de 313 tareas del Sprint, 89 son de Bryan terminadas, 22 de Catalina (HU-142 y HU-143) y ninguna de Emilio. El equipo acuerda que el Sprint 6 se planifica sobre lo que cada uno puede sostener de verdad, y que las historias bloqueantes del Sprint 4 (HU-082, HU-091, HU-097) entran primero. Dejamos constancia de algo que se ve en las fechas: vamos adelantados respecto del calendario. SIGMA son 785 puntos, 138 historias y 20 épicas para un equipo de tres, y la única forma de absorber ese alcance fue adelantar construcción: lo que aquí se registra en la ventana del Sprint 4 y del Sprint 5 quedó construido y verificado contra la base entre el 11 y el 14 de septiembre. El registro mantiene el calendario planificado para no romper la trazabilidad con el Sprint Backlog, el burndown y los informes de prueba. REPARTO PARA TERMINAR EL SPRINT 5: cada historia la hace UNA persona de punta a punta —desarrollo, pruebas, documentación y validación—, y las que tocan el mismo código van juntas: Bryan HU-117 y HU-125 (la orden), Catalina ya cerró HU-142 y HU-143 (Archivo_Vinculo), Emilio HU-131 y HU-162.</t>
         </is>
       </c>
     </row>

</xml_diff>